<commit_message>
se agregaron varios archivos
</commit_message>
<xml_diff>
--- a/docs/EBS Item Templates_08282026.xlsx
+++ b/docs/EBS Item Templates_08282026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JCCC\ArGlobal-1\CreateItemApp\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JCCC\ArGlobal-1\Create-item-App\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0EACE06-AA7C-45FF-BD7F-205582C2CCFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C903E7ED-9EC1-4FEE-BFE1-8C0B1BD0212D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{F92D7170-3C54-44E9-9CC4-7EEC395E8CC2}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1814" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1816" uniqueCount="379">
   <si>
     <t>ADHESIVES</t>
   </si>
@@ -1176,13 +1176,19 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>MH-94904-1012</t>
+  </si>
+  <si>
+    <t>MH-94904-1013</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1194,6 +1200,14 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Carlito"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1238,7 +1252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1259,6 +1273,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6685,11 +6700,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E210809-C76C-4E6B-BCDE-B6672DB11A2B}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="13.9140625" customWidth="1"/>
+    <col min="1" max="1" width="21.75" customWidth="1"/>
     <col min="2" max="2" width="7.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="4" bestFit="1" customWidth="1"/>
@@ -7057,7 +7071,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="15" spans="1:10" hidden="1">
+    <row r="15" spans="1:10">
       <c r="A15" t="s">
         <v>335</v>
       </c>
@@ -7070,8 +7084,14 @@
       <c r="F15" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" hidden="1">
+      <c r="G15" t="s">
+        <v>377</v>
+      </c>
+      <c r="I15">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
       <c r="A16" t="s">
         <v>335</v>
       </c>
@@ -7084,8 +7104,14 @@
       <c r="F16" t="s">
         <v>338</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="15" hidden="1" customHeight="1">
+      <c r="G16" t="s">
+        <v>378</v>
+      </c>
+      <c r="I16">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="15" customHeight="1">
       <c r="A17" s="1" t="s">
         <v>339</v>
       </c>
@@ -7102,7 +7128,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="18" spans="1:6" ht="15" customHeight="1">
       <c r="A18" s="1" t="s">
         <v>339</v>
       </c>
@@ -7119,7 +7145,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="19" spans="1:6" ht="15" customHeight="1">
       <c r="A19" s="1" t="s">
         <v>339</v>
       </c>
@@ -7139,7 +7165,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="20" spans="1:6" ht="15" customHeight="1">
       <c r="A20" s="1" t="s">
         <v>339</v>
       </c>
@@ -7156,7 +7182,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="21" spans="1:6" ht="15" customHeight="1">
       <c r="A21" s="1" t="s">
         <v>339</v>
       </c>
@@ -7173,7 +7199,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="22" spans="1:6" ht="15" customHeight="1">
       <c r="A22" s="1" t="s">
         <v>339</v>
       </c>
@@ -7190,7 +7216,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="23" spans="1:6" ht="15" customHeight="1">
       <c r="A23" s="1" t="s">
         <v>339</v>
       </c>
@@ -7206,8 +7232,9 @@
       <c r="E23" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" ht="15" hidden="1" customHeight="1">
+      <c r="F23" s="8"/>
+    </row>
+    <row r="24" spans="1:6" ht="15" customHeight="1">
       <c r="A24" s="1" t="s">
         <v>339</v>
       </c>
@@ -7224,7 +7251,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="25" spans="1:6" ht="15" customHeight="1">
       <c r="A25" s="1" t="s">
         <v>339</v>
       </c>
@@ -7241,7 +7268,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="26" spans="1:6" ht="15" customHeight="1">
       <c r="A26" s="1" t="s">
         <v>339</v>
       </c>
@@ -7261,7 +7288,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="27" spans="1:6" ht="15" customHeight="1">
       <c r="A27" s="1" t="s">
         <v>339</v>
       </c>
@@ -7278,7 +7305,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="28" spans="1:6" ht="15" customHeight="1">
       <c r="A28" s="1" t="s">
         <v>339</v>
       </c>
@@ -7295,7 +7322,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="29" spans="1:6" ht="15" customHeight="1">
       <c r="A29" s="1" t="s">
         <v>339</v>
       </c>
@@ -7312,7 +7339,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="30" spans="1:6" ht="15" customHeight="1">
       <c r="A30" s="1" t="s">
         <v>343</v>
       </c>
@@ -7329,7 +7356,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="31" spans="1:6" ht="15" customHeight="1">
       <c r="A31" s="1" t="s">
         <v>343</v>
       </c>
@@ -7346,7 +7373,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="32" spans="1:6" ht="15" customHeight="1">
       <c r="A32" s="1" t="s">
         <v>343</v>
       </c>
@@ -7363,7 +7390,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="33" spans="1:6" ht="15" customHeight="1">
       <c r="A33" s="1" t="s">
         <v>343</v>
       </c>
@@ -7380,7 +7407,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="34" spans="1:6" ht="15" customHeight="1">
       <c r="A34" s="1" t="s">
         <v>343</v>
       </c>
@@ -7397,7 +7424,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="35" spans="1:6" ht="15" customHeight="1">
       <c r="A35" s="1" t="s">
         <v>343</v>
       </c>
@@ -7414,7 +7441,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="36" spans="1:6" ht="15" customHeight="1">
       <c r="A36" s="1" t="s">
         <v>343</v>
       </c>
@@ -7431,7 +7458,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="37" spans="1:6" ht="15" customHeight="1">
       <c r="A37" s="1" t="s">
         <v>343</v>
       </c>
@@ -7448,7 +7475,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="38" spans="1:6" ht="15" customHeight="1">
       <c r="A38" s="1" t="s">
         <v>343</v>
       </c>
@@ -7465,7 +7492,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="39" spans="1:6" ht="15" customHeight="1">
       <c r="A39" s="1" t="s">
         <v>343</v>
       </c>
@@ -7482,7 +7509,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="40" spans="1:6" ht="15" customHeight="1">
       <c r="A40" s="1" t="s">
         <v>343</v>
       </c>
@@ -7499,7 +7526,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="41" spans="1:6" ht="15" customHeight="1">
       <c r="A41" s="1" t="s">
         <v>343</v>
       </c>
@@ -7516,7 +7543,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="42" spans="1:6" ht="15" customHeight="1">
       <c r="A42" s="1" t="s">
         <v>343</v>
       </c>
@@ -7533,7 +7560,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="43" spans="1:6" ht="15" customHeight="1">
       <c r="A43" s="2" t="s">
         <v>147</v>
       </c>
@@ -7547,7 +7574,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="44" spans="1:6" ht="15" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>345</v>
       </c>
@@ -7558,7 +7585,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="15" hidden="1" customHeight="1">
+    <row r="45" spans="1:6" ht="15" customHeight="1">
       <c r="A45" s="2" t="s">
         <v>347</v>
       </c>
@@ -7570,14 +7597,9 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J45" xr:uid="{8E210809-C76C-4E6B-BCDE-B6672DB11A2B}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Adhesive Coating"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:J45" xr:uid="{8E210809-C76C-4E6B-BCDE-B6672DB11A2B}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Se establecio nueva configuración de carpetas y estructura de archivos
</commit_message>
<xml_diff>
--- a/docs/EBS Item Templates_08282026.xlsx
+++ b/docs/EBS Item Templates_08282026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JCCC\ArGlobal-1\Create-item-App\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C903E7ED-9EC1-4FEE-BFE1-8C0B1BD0212D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{428A7D3B-25C9-4947-A4DA-9741F3B13797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{F92D7170-3C54-44E9-9CC4-7EEC395E8CC2}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1816" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1833" uniqueCount="396">
   <si>
     <t>ADHESIVES</t>
   </si>
@@ -1182,6 +1182,57 @@
   </si>
   <si>
     <t>MH-94904-1013</t>
+  </si>
+  <si>
+    <t>MH-94904-1014</t>
+  </si>
+  <si>
+    <t>MH-94904-1015</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> MH-94904-1016</t>
+  </si>
+  <si>
+    <t>MH-94904-1017</t>
+  </si>
+  <si>
+    <t>MH-94904-1018</t>
+  </si>
+  <si>
+    <t>MH-94904-1019</t>
+  </si>
+  <si>
+    <t>MH-94904-1020</t>
+  </si>
+  <si>
+    <t>MH-94904-1021</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> MH-94904-1022</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> MH-94904-1023</t>
+  </si>
+  <si>
+    <t>MH-94904-1024</t>
+  </si>
+  <si>
+    <t>MH-94904-1025</t>
+  </si>
+  <si>
+    <t>MH-94904-1026</t>
+  </si>
+  <si>
+    <t>MH-94904-1027</t>
+  </si>
+  <si>
+    <t>MH-94904-1028</t>
+  </si>
+  <si>
+    <t>MH-94904-1029</t>
+  </si>
+  <si>
+    <t>MH-94904-1030</t>
   </si>
 </sst>
 </file>
@@ -1746,15 +1797,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98219B57-BFDA-47C0-9733-31F625450BED}">
   <dimension ref="A1:Z104"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="43.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.4140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22.75" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.58203125" customWidth="1"/>
+    <col min="8" max="8" width="19.625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26">
@@ -6471,7 +6522,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC84ADCB-CE70-4C75-9B3D-B14D791A02F8}">
   <dimension ref="B3:V61"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.625" defaultRowHeight="14.25"/>
   <sheetData>
     <row r="3" spans="2:22">
       <c r="B3" t="s">
@@ -6700,22 +6751,23 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E210809-C76C-4E6B-BCDE-B6672DB11A2B}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:J45"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.625" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="21.75" customWidth="1"/>
-    <col min="2" max="2" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.1640625" customWidth="1"/>
+    <col min="5" max="5" width="28.125" customWidth="1"/>
     <col min="6" max="6" width="9" customWidth="1"/>
-    <col min="7" max="7" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
-    <col min="9" max="9" width="8.4140625" customWidth="1"/>
-    <col min="10" max="10" width="44.9140625" customWidth="1"/>
+    <col min="9" max="9" width="13.5" customWidth="1"/>
+    <col min="10" max="10" width="44.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="35.5" customHeight="1">
+    <row r="1" spans="1:10" ht="35.450000000000003" customHeight="1">
       <c r="A1" s="6" t="s">
         <v>303</v>
       </c>
@@ -6747,7 +6799,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" hidden="1">
       <c r="A2" t="s">
         <v>307</v>
       </c>
@@ -6776,7 +6828,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" hidden="1">
       <c r="A3" t="s">
         <v>307</v>
       </c>
@@ -6805,7 +6857,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" hidden="1">
       <c r="A4" t="s">
         <v>307</v>
       </c>
@@ -6826,7 +6878,7 @@
       </c>
       <c r="I4" s="5"/>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" hidden="1">
       <c r="A5" t="s">
         <v>307</v>
       </c>
@@ -6855,7 +6907,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="56">
+    <row r="6" spans="1:10" ht="57" hidden="1">
       <c r="A6" t="s">
         <v>307</v>
       </c>
@@ -6887,7 +6939,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" hidden="1">
       <c r="A7" t="s">
         <v>307</v>
       </c>
@@ -6908,7 +6960,7 @@
       </c>
       <c r="I7" s="5"/>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" hidden="1">
       <c r="A8" t="s">
         <v>307</v>
       </c>
@@ -6929,7 +6981,7 @@
       </c>
       <c r="I8" s="5"/>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" hidden="1">
       <c r="A9" t="s">
         <v>307</v>
       </c>
@@ -6950,7 +7002,7 @@
       </c>
       <c r="I9" s="5"/>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" hidden="1">
       <c r="A10" t="s">
         <v>307</v>
       </c>
@@ -6979,7 +7031,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" hidden="1">
       <c r="A11" t="s">
         <v>307</v>
       </c>
@@ -7000,7 +7052,7 @@
       </c>
       <c r="I11" s="5"/>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" hidden="1">
       <c r="A12" t="s">
         <v>307</v>
       </c>
@@ -7021,7 +7073,7 @@
       </c>
       <c r="I12" s="5"/>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" hidden="1">
       <c r="A13" t="s">
         <v>307</v>
       </c>
@@ -7042,7 +7094,7 @@
       </c>
       <c r="I13" s="5"/>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" hidden="1">
       <c r="A14" t="s">
         <v>307</v>
       </c>
@@ -7071,7 +7123,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" hidden="1">
       <c r="A15" t="s">
         <v>335</v>
       </c>
@@ -7087,11 +7139,14 @@
       <c r="G15" t="s">
         <v>377</v>
       </c>
+      <c r="H15" s="3">
+        <v>46265</v>
+      </c>
       <c r="I15">
         <v>106</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" hidden="1">
       <c r="A16" t="s">
         <v>335</v>
       </c>
@@ -7107,11 +7162,14 @@
       <c r="G16" t="s">
         <v>378</v>
       </c>
+      <c r="H16" s="3">
+        <v>46265</v>
+      </c>
       <c r="I16">
         <v>105</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="15" customHeight="1">
+    <row r="17" spans="1:9" ht="15" customHeight="1">
       <c r="A17" s="1" t="s">
         <v>339</v>
       </c>
@@ -7127,8 +7185,17 @@
       <c r="E17" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" ht="15" customHeight="1">
+      <c r="G17" t="s">
+        <v>379</v>
+      </c>
+      <c r="H17" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I17" s="5">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="15" customHeight="1">
       <c r="A18" s="1" t="s">
         <v>339</v>
       </c>
@@ -7144,8 +7211,17 @@
       <c r="E18" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="15" customHeight="1">
+      <c r="G18" t="s">
+        <v>380</v>
+      </c>
+      <c r="H18" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I18">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="15" customHeight="1">
       <c r="A19" s="1" t="s">
         <v>339</v>
       </c>
@@ -7164,8 +7240,11 @@
       <c r="F19" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" ht="15" customHeight="1">
+      <c r="H19" s="3">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="15" customHeight="1">
       <c r="A20" s="1" t="s">
         <v>339</v>
       </c>
@@ -7181,8 +7260,17 @@
       <c r="E20" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" ht="15" customHeight="1">
+      <c r="G20" t="s">
+        <v>381</v>
+      </c>
+      <c r="H20" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I20">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="15" hidden="1" customHeight="1">
       <c r="A21" s="1" t="s">
         <v>339</v>
       </c>
@@ -7198,8 +7286,9 @@
       <c r="E21" t="s">
         <v>342</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="15" customHeight="1">
+      <c r="H21" s="3"/>
+    </row>
+    <row r="22" spans="1:9" ht="15" customHeight="1">
       <c r="A22" s="1" t="s">
         <v>339</v>
       </c>
@@ -7215,8 +7304,17 @@
       <c r="E22" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" ht="15" customHeight="1">
+      <c r="G22" t="s">
+        <v>382</v>
+      </c>
+      <c r="H22" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I22">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="15" customHeight="1">
       <c r="A23" s="1" t="s">
         <v>339</v>
       </c>
@@ -7233,8 +7331,17 @@
         <v>11</v>
       </c>
       <c r="F23" s="8"/>
-    </row>
-    <row r="24" spans="1:6" ht="15" customHeight="1">
+      <c r="G23" t="s">
+        <v>383</v>
+      </c>
+      <c r="H23" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I23">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="15" hidden="1" customHeight="1">
       <c r="A24" s="1" t="s">
         <v>339</v>
       </c>
@@ -7250,8 +7357,9 @@
       <c r="E24" t="s">
         <v>332</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" ht="15" customHeight="1">
+      <c r="H24" s="3"/>
+    </row>
+    <row r="25" spans="1:9" ht="15" customHeight="1">
       <c r="A25" s="1" t="s">
         <v>339</v>
       </c>
@@ -7267,8 +7375,17 @@
       <c r="E25" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" ht="15" customHeight="1">
+      <c r="G25" t="s">
+        <v>384</v>
+      </c>
+      <c r="H25" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I25">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="15" customHeight="1">
       <c r="A26" s="1" t="s">
         <v>339</v>
       </c>
@@ -7287,8 +7404,17 @@
       <c r="F26" t="s">
         <v>341</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" ht="15" customHeight="1">
+      <c r="G26" t="s">
+        <v>385</v>
+      </c>
+      <c r="H26" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I26">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="15" hidden="1" customHeight="1">
       <c r="A27" s="1" t="s">
         <v>339</v>
       </c>
@@ -7304,8 +7430,9 @@
       <c r="E27" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" ht="15" customHeight="1">
+      <c r="H27" s="3"/>
+    </row>
+    <row r="28" spans="1:9" ht="15" hidden="1" customHeight="1">
       <c r="A28" s="1" t="s">
         <v>339</v>
       </c>
@@ -7321,8 +7448,9 @@
       <c r="E28" t="s">
         <v>332</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" ht="15" customHeight="1">
+      <c r="H28" s="3"/>
+    </row>
+    <row r="29" spans="1:9" ht="15" customHeight="1">
       <c r="A29" s="1" t="s">
         <v>339</v>
       </c>
@@ -7338,8 +7466,17 @@
       <c r="E29" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" ht="15" customHeight="1">
+      <c r="G29" t="s">
+        <v>386</v>
+      </c>
+      <c r="H29" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I29">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="15" customHeight="1">
       <c r="A30" s="1" t="s">
         <v>343</v>
       </c>
@@ -7355,8 +7492,17 @@
       <c r="E30" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" ht="15" customHeight="1">
+      <c r="G30" t="s">
+        <v>387</v>
+      </c>
+      <c r="H30" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I30">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="15" customHeight="1">
       <c r="A31" s="1" t="s">
         <v>343</v>
       </c>
@@ -7372,8 +7518,17 @@
       <c r="E31" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" ht="15" customHeight="1">
+      <c r="G31" t="s">
+        <v>388</v>
+      </c>
+      <c r="H31" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I31">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="15" hidden="1" customHeight="1">
       <c r="A32" s="1" t="s">
         <v>343</v>
       </c>
@@ -7389,8 +7544,9 @@
       <c r="E32" t="s">
         <v>332</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" ht="15" customHeight="1">
+      <c r="H32" s="3"/>
+    </row>
+    <row r="33" spans="1:9" ht="15" customHeight="1">
       <c r="A33" s="1" t="s">
         <v>343</v>
       </c>
@@ -7406,8 +7562,17 @@
       <c r="E33" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" ht="15" customHeight="1">
+      <c r="G33" t="s">
+        <v>389</v>
+      </c>
+      <c r="H33" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I33">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="15" customHeight="1">
       <c r="A34" s="1" t="s">
         <v>343</v>
       </c>
@@ -7423,8 +7588,11 @@
       <c r="E34" t="s">
         <v>342</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" ht="15" customHeight="1">
+      <c r="H34" s="3">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="15" customHeight="1">
       <c r="A35" s="1" t="s">
         <v>343</v>
       </c>
@@ -7440,8 +7608,17 @@
       <c r="E35" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" ht="15" customHeight="1">
+      <c r="G35" t="s">
+        <v>390</v>
+      </c>
+      <c r="H35" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I35">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="15" customHeight="1">
       <c r="A36" s="1" t="s">
         <v>343</v>
       </c>
@@ -7457,8 +7634,17 @@
       <c r="E36" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" ht="15" customHeight="1">
+      <c r="G36" t="s">
+        <v>391</v>
+      </c>
+      <c r="H36" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I36">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="15" hidden="1" customHeight="1">
       <c r="A37" s="1" t="s">
         <v>343</v>
       </c>
@@ -7474,8 +7660,9 @@
       <c r="E37" t="s">
         <v>332</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" ht="15" customHeight="1">
+      <c r="H37" s="3"/>
+    </row>
+    <row r="38" spans="1:9" ht="15" customHeight="1">
       <c r="A38" s="1" t="s">
         <v>343</v>
       </c>
@@ -7491,8 +7678,17 @@
       <c r="E38" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" ht="15" customHeight="1">
+      <c r="G38" t="s">
+        <v>392</v>
+      </c>
+      <c r="H38" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I38">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="15" customHeight="1">
       <c r="A39" s="1" t="s">
         <v>343</v>
       </c>
@@ -7508,8 +7704,17 @@
       <c r="E39" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" ht="15" customHeight="1">
+      <c r="G39" t="s">
+        <v>393</v>
+      </c>
+      <c r="H39" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I39">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="15" hidden="1" customHeight="1">
       <c r="A40" s="1" t="s">
         <v>343</v>
       </c>
@@ -7525,8 +7730,9 @@
       <c r="E40" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" ht="15" customHeight="1">
+      <c r="H40" s="3"/>
+    </row>
+    <row r="41" spans="1:9" ht="15" hidden="1" customHeight="1">
       <c r="A41" s="1" t="s">
         <v>343</v>
       </c>
@@ -7542,8 +7748,9 @@
       <c r="E41" t="s">
         <v>332</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" ht="15" customHeight="1">
+      <c r="H41" s="3"/>
+    </row>
+    <row r="42" spans="1:9" ht="15" customHeight="1">
       <c r="A42" s="1" t="s">
         <v>343</v>
       </c>
@@ -7559,8 +7766,17 @@
       <c r="E42" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" ht="15" customHeight="1">
+      <c r="G42" t="s">
+        <v>394</v>
+      </c>
+      <c r="H42" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I42">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="15" customHeight="1">
       <c r="A43" s="2" t="s">
         <v>147</v>
       </c>
@@ -7573,8 +7789,17 @@
       <c r="F43" t="s">
         <v>344</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" ht="15" customHeight="1">
+      <c r="G43" t="s">
+        <v>395</v>
+      </c>
+      <c r="H43" s="3">
+        <v>46266</v>
+      </c>
+      <c r="I43">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="15" hidden="1" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>345</v>
       </c>
@@ -7585,7 +7810,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="15" customHeight="1">
+    <row r="45" spans="1:9" ht="15" hidden="1" customHeight="1">
       <c r="A45" s="2" t="s">
         <v>347</v>
       </c>
@@ -7597,7 +7822,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J45" xr:uid="{8E210809-C76C-4E6B-BCDE-B6672DB11A2B}"/>
+  <autoFilter ref="A1:J45" xr:uid="{8E210809-C76C-4E6B-BCDE-B6672DB11A2B}">
+    <filterColumn colId="7">
+      <filters>
+        <dateGroupItem year="2026" month="9" dateTimeGrouping="month"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -7606,10 +7837,10 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6DADA09-45D8-4886-8D6A-309F3B7584C3}">
   <dimension ref="A2:C10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.625" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="17.25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.58203125" customWidth="1"/>
+    <col min="2" max="2" width="10.625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:3">

</xml_diff>